<commit_message>
📊 Horarios actualizados Línea 141 - 4238
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:07:09</t>
+          <t>Última actualización: 00:49:19</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:07:09</t>
+          <t>00:49:19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>00:07:09</t>
+          <t>00:49:19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:07:09</t>
+          <t>Última actualización: 00:49:19</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:07:09</t>
+          <t>00:49:19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:07:09</t>
+          <t>Última actualización: 00:49:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4239
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:19</t>
+          <t>Última actualización: 01:14:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -498,23 +498,73 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>01:14:46</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01:58</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>44</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>00:49:19</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>01:59</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>70</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>01:14:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>102</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:19</t>
+          <t>Última actualización: 01:14:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -602,6 +652,31 @@
         <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>01:14:46</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>102</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -631,7 +706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:19</t>
+          <t>Última actualización: 01:14:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4240
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:14:46</t>
+          <t>Última actualización: 01:47:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -565,6 +565,31 @@
         <v>102</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>01:47:05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>03:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>75</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -594,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:14:46</t>
+          <t>Última actualización: 01:47:05</t>
         </is>
       </c>
     </row>
@@ -706,7 +731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:14:46</t>
+          <t>Última actualización: 01:47:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4241
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:05</t>
+          <t>Última actualización: 02:03:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -573,23 +573,98 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>02:03:54</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>03:01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>58</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>01:47:05</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>03:02</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>75</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>02:03:54</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>105</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>02:03:54</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>118</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -619,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:05</t>
+          <t>Última actualización: 02:03:54</t>
         </is>
       </c>
     </row>
@@ -731,7 +806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:05</t>
+          <t>Última actualización: 02:03:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4242
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:54</t>
+          <t>Última actualización: 02:34:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>01:47:05</t>
+          <t>02:34:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>02:03:54</t>
+          <t>02:34:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -665,6 +665,31 @@
         <v>118</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>02:34:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>88</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -694,7 +719,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:54</t>
+          <t>Última actualización: 02:34:00</t>
         </is>
       </c>
     </row>
@@ -806,7 +831,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:54</t>
+          <t>Última actualización: 02:34:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4243
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:34:00</t>
+          <t>Última actualización: 02:54:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:03:54</t>
+          <t>02:54:46</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>02:34:00</t>
+          <t>02:54:46</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>02:03:54</t>
+          <t>02:54:46</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>118</v>
+        <v>67</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -690,6 +690,56 @@
         <v>88</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>02:54:46</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>113</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>02:54:46</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>119</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -719,7 +769,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:34:00</t>
+          <t>Última actualización: 02:54:46</t>
         </is>
       </c>
     </row>
@@ -831,7 +881,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:34:00</t>
+          <t>Última actualización: 02:54:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4244
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:54:46</t>
+          <t>Última actualización: 03:17:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>02:54:46</t>
+          <t>03:17:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>02:34:00</t>
+          <t>03:17:21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>88</v>
+        <v>45</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,23 +723,48 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>02:54:46</t>
+          <t>03:17:21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>91</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>03:17:21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>04:53</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>119</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="n">
+        <v>96</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -769,7 +794,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:54:46</t>
+          <t>Última actualización: 03:17:21</t>
         </is>
       </c>
     </row>
@@ -881,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:54:46</t>
+          <t>Última actualización: 03:17:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4245
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:17:21</t>
+          <t>Última actualización: 03:59:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>03:17:21</t>
+          <t>03:59:22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>03:17:21</t>
+          <t>03:59:22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>03:17:21</t>
+          <t>03:59:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -762,9 +762,109 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03:59:22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>78</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>03:59:22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>83</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>03:59:22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>05:39</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>03:59:22</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>108</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -794,7 +894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:17:21</t>
+          <t>Última actualización: 03:59:22</t>
         </is>
       </c>
     </row>
@@ -906,7 +1006,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:17:21</t>
+          <t>Última actualización: 03:59:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4246
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:59:22</t>
+          <t>Última actualización: 04:29:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -848,23 +848,123 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:29:01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>05:47</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>108</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>78</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:29:01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>92</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:29:01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:29:01</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>104</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:59:22</t>
+          <t>Última actualización: 04:29:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -977,6 +1077,31 @@
         <v>102</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:29:01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:13</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>104</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1006,7 +1131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:59:22</t>
+          <t>Última actualización: 04:29:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4247
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:29:01</t>
+          <t>Última actualización: 04:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,23 +948,173 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>81</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>04:29:01</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>06:13</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>104</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>99</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>103</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>108</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>108</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>110</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,14 +1144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:29:01</t>
+          <t>Última actualización: 04:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1085,23 +1235,48 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>04:51:36</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>04:29:01</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>06:13</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>104</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1131,7 +1306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:29:01</t>
+          <t>Última actualización: 04:51:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4248
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:36</t>
+          <t>Última actualización: 05:13:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:59:22</t>
+          <t>04:51:36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05:39</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>05:24</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>03:59:22</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>05:39</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -953,16 +953,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>99</v>
+        <v>56</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:13</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,23 +1098,173 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>81</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>86</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>86</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>87</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>04:51:36</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>06:41</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D35" t="n">
         <v>110</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>102</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>106</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1131,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1144,14 +1294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:36</t>
+          <t>Última actualización: 05:13:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1385,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1249,7 +1399,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1277,6 +1427,31 @@
         <v>104</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:13:43</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>102</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1306,7 +1481,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:36</t>
+          <t>Última actualización: 05:13:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4249
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:13:43</t>
+          <t>Última actualización: 05:45:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>05:45</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,12 +1048,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:29:01</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>104</v>
+        <v>27</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>04:29:01</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:13</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,12 +1198,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>04:51:36</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,23 +1248,198 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>70</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>06:59</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>106</v>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="n">
+        <v>74</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>94</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>95</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>96</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>101</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>110</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>112</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1281,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1294,14 +1469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:13:43</t>
+          <t>Última actualización: 05:45:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1399,7 +1574,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1435,7 +1610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>05:45:20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1449,9 +1624,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>102</v>
+        <v>70</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1468,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1481,14 +1681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:13:43</t>
+          <t>Última actualización: 05:45:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -1539,6 +1739,31 @@
         <v>10</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:45:20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>119</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4250
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:45:20</t>
+          <t>Última actualización: 06:02:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,9 +1437,59 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06:02:21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>113</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06:02:21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>114</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1469,7 +1519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:45:20</t>
+          <t>Última actualización: 06:02:21</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1610,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1574,7 +1624,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1610,7 +1660,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1624,7 +1674,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1635,7 +1685,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1649,7 +1699,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1681,7 +1731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:45:20</t>
+          <t>Última actualización: 06:02:21</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1797,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:45:20</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1761,7 +1811,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4251
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:02:21</t>
+          <t>Última actualización: 06:34:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>05:13:43</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>87</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,12 +1223,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>05:13:43</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,23 +1473,248 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>61</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>62</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>06:02:21</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>95</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>81</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:02:21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>07:56</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D50" t="n">
         <v>114</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>85</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>97</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>103</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>107</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>114</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1506,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1519,14 +1744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:02:21</t>
+          <t>Última actualización: 06:34:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1885,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1674,7 +1899,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1685,23 +1910,73 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>45</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>06:02:21</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>07:20</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>78</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>60</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1718,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1731,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:02:21</t>
+          <t>Última actualización: 06:34:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1797,7 +2072,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1811,9 +2086,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>102</v>
+        <v>70</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:34:33</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>119</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4252
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:34:34</t>
+          <t>Última actualización: 06:52:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,12 +1523,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>95</v>
+        <v>44</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,12 +1598,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,23 +1698,148 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>85</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>89</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>08:28</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>114</v>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D57" t="n">
+        <v>96</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>106</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>109</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>109</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1731,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1744,14 +1869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:34:34</t>
+          <t>Última actualización: 06:52:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1885,7 +2010,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1899,7 +2024,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1910,7 +2035,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1924,7 +2049,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1960,7 +2085,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1974,9 +2099,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>106</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:34:34</t>
+          <t>Última actualización: 06:52:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2222,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2086,7 +2236,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2097,7 +2247,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2111,11 +2261,36 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>116</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4253
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:27</t>
+          <t>Última actualización: 07:10:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:18</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,12 +1423,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,23 +1823,298 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>67</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>71</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>77</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>06:52:27</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>96</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>87</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>106</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>90</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>08:41</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>91</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="D68" t="n">
         <v>109</v>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>104</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>106</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>116</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1856,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1869,14 +2144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:27</t>
+          <t>Última actualización: 07:10:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2310,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2049,7 +2324,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2085,7 +2360,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2099,7 +2374,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2110,23 +2385,98 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>87</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>06:52:27</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>106</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>106</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2143,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2156,14 +2506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:52:27</t>
+          <t>Última actualización: 07:10:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -2222,12 +2572,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2236,7 +2586,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2252,7 +2602,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2261,7 +2611,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2272,23 +2622,98 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>06:52:27</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>101</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:10:54</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>97</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:52:27</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>08:48</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D12" t="n">
         <v>116</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4254
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:54</t>
+          <t>Última actualización: 07:39:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 72</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:39</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>114</v>
+        <v>16</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>49</v>
+        <v>114</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:27</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>106</v>
+        <v>49</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,12 +2023,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,23 +2098,173 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>75</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>77</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>09:06</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>116</v>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D73" t="n">
+        <v>87</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>92</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>98</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>100</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>07:39:30</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>107</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2144,7 +2294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:54</t>
+          <t>Última actualización: 07:39:30</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2560,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2424,7 +2574,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2435,7 +2585,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2449,7 +2599,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2460,7 +2610,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2474,7 +2624,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2506,7 +2656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:10:54</t>
+          <t>Última actualización: 07:39:30</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2747,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2611,7 +2761,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2647,7 +2797,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2661,7 +2811,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2697,7 +2847,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2711,7 +2861,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4255
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:39:30</t>
+          <t>Última actualización: 07:54:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 72</t>
+          <t>Total filas: 77</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1823,12 +1823,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:27</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,12 +1948,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,12 +1998,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2253,18 +2253,143 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>100</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>87</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
           <t>09:26</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D79" t="n">
+        <v>92</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>104</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
         <v>107</v>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>109</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2294,7 +2419,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:39:30</t>
+          <t>Última actualización: 07:54:48</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2660,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2549,7 +2674,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2585,7 +2710,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2599,7 +2724,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2610,7 +2735,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2624,7 +2749,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2643,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2656,14 +2781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:39:30</t>
+          <t>Última actualización: 07:54:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2897,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2786,7 +2911,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2822,7 +2947,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2836,7 +2961,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2866,6 +2991,31 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:54:48</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>93</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4256
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:54:48</t>
+          <t>Última actualización: 08:08:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 77</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,12 +2273,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,23 +2373,148 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>90</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>93</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>09:43</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D84" t="n">
+        <v>95</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>108</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
         <v>109</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>113</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2406,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2419,14 +2544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:54:48</t>
+          <t>Última actualización: 08:08:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2785,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2674,7 +2799,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2710,7 +2835,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2724,7 +2849,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2735,7 +2860,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2749,9 +2874,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>109</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2768,7 +2918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2781,14 +2931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:54:48</t>
+          <t>Última actualización: 08:08:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -2897,7 +3047,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2911,7 +3061,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2947,7 +3097,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2961,7 +3111,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2997,7 +3147,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3011,11 +3161,36 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>119</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4257
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:08:42</t>
+          <t>Última actualización: 08:30:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 91</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:58</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,16 +2228,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,12 +2273,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,12 +2298,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>108</v>
+        <v>68</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,23 +2498,248 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>73</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>86</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
           <t>08:08:42</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>109</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>88</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>89</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08:08:42</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t>10:01</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>23_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D92" t="n">
         <v>113</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>99</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>103</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>116</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>117</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2531,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,14 +2769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:08:42</t>
+          <t>Última actualización: 08:30:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2810,7 +3035,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2824,7 +3049,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2835,7 +3060,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2849,7 +3074,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2860,7 +3085,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2874,7 +3099,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2902,6 +3127,31 @@
         <v>109</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>88</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2918,7 +3168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2931,14 +3181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:08:42</t>
+          <t>Última actualización: 08:30:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -3047,12 +3297,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08:32</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3061,7 +3311,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -3072,12 +3322,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3086,7 +3336,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -3097,37 +3347,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08:47</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:47</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3136,7 +3386,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -3147,25 +3397,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -3177,18 +3427,68 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>79</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>58</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:30:35</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>10:07</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>119</v>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4258
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:30:35</t>
+          <t>Última actualización: 08:49:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 91</t>
+          <t>Total filas: 96</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>113</v>
+        <v>72</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>116</v>
+        <v>84</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,23 +2723,148 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>96</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
           <t>08:30:35</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>116</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
         <is>
           <t>10:27</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>117</v>
-      </c>
-      <c r="E96" t="inlineStr">
+      <c r="D98" t="n">
+        <v>98</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>106</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>114</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>115</v>
+      </c>
+      <c r="E101" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2769,7 +2894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:30:35</t>
+          <t>Última actualización: 08:49:51</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3185,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3074,7 +3199,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3085,7 +3210,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3099,7 +3224,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3110,7 +3235,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3124,7 +3249,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3168,7 +3293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3181,14 +3306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:30:35</t>
+          <t>Última actualización: 08:49:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3422,37 +3547,37 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>08:49</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3461,7 +3586,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3477,20 +3602,95 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>58</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>10:07</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>97</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="n">
+        <v>78</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>98</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>105</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4259
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:51</t>
+          <t>Última actualización: 08:59:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 96</t>
+          <t>Total filas: 102</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2248,12 +2248,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,12 +2298,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,12 +2348,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:39:30</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:54:48</t>
+          <t>07:39:30</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>07:54:48</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,12 +2623,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>10:35</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,23 +2848,173 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
+          <t>08:59:52</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>88</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>08:49:51</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>106</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>08:59:52</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>104</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>08:59:52</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>104</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
         <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D101" t="n">
+      <c r="D105" t="n">
         <v>115</v>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08:59:52</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>117</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08:59:52</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>119</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2894,7 +3044,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:51</t>
+          <t>Última actualización: 08:59:52</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3385,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3249,7 +3399,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3306,7 +3456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:49:51</t>
+          <t>Última actualización: 08:59:52</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3722,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3586,7 +3736,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3622,7 +3772,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3636,7 +3786,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3647,7 +3797,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3661,7 +3811,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3672,7 +3822,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3686,7 +3836,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4260
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E107"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:59:52</t>
+          <t>Última actualización: 09:36:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 102</t>
+          <t>Total filas: 112</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2473,12 +2473,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:37</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,12 +2673,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,16 +2703,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>10:35</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:27</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>104</v>
+        <v>51</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2953,16 +2953,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:35</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,23 +2998,273 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>67</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08:49:51</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>115</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>80</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
           <t>10:58</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D107" t="n">
-        <v>119</v>
-      </c>
-      <c r="E107" t="inlineStr">
+      <c r="D110" t="n">
+        <v>82</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>86</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>88</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>94</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>97</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>102</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>111</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>118</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3031,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3044,14 +3294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:59:52</t>
+          <t>Última actualización: 09:36:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3635,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3399,7 +3649,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3427,6 +3677,31 @@
         <v>88</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>111</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3443,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3456,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:59:52</t>
+          <t>Última actualización: 09:36:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3772,7 +4047,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3786,7 +4061,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3797,7 +4072,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3811,7 +4086,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3822,7 +4097,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3836,11 +4111,36 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>111</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4261
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:36:56</t>
+          <t>Última actualización: 10:11:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 112</t>
+          <t>Total filas: 124</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>116</v>
+        <v>15</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:37</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>115</v>
+        <v>32</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>86</v>
+        <v>45</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>102</v>
+        <v>57</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>111</v>
+        <v>59</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,23 +3248,323 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>62</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>09:36:56</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>97</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>63</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>102</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>69</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>74</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>76</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
         <is>
           <t>11:34</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D117" t="n">
+      <c r="D124" t="n">
         <v>118</v>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>87</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>90</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>102</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>107</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>117</v>
+      </c>
+      <c r="E129" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3281,7 +3581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3294,14 +3594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:36:56</t>
+          <t>Última actualización: 10:11:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3985,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3699,9 +3999,34 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>87</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3731,7 +4056,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:36:56</t>
+          <t>Última actualización: 10:11:42</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4397,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4086,7 +4411,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4097,7 +4422,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4111,7 +4436,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -4122,7 +4447,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4136,7 +4461,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4262
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:11:42</t>
+          <t>Última actualización: 10:43:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 124</t>
+          <t>Total filas: 139</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:46</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>102</v>
+        <v>27</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>118</v>
+        <v>63</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>107</v>
+        <v>69</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,23 +3548,398 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>42</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>44</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>09:36:56</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>118</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>55</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
           <t>10:11:42</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>90</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>61</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>69</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>102</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>74</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>10:11:42</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>107</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
         <is>
           <t>12:08</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D129" t="n">
-        <v>117</v>
-      </c>
-      <c r="E129" t="inlineStr">
+      <c r="D139" t="n">
+        <v>85</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>92</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>104</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>113</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>115</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>119</v>
+      </c>
+      <c r="E144" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3581,7 +3956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3594,14 +3969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:11:42</t>
+          <t>Última actualización: 10:43:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3985,7 +4360,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3999,7 +4374,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4010,7 +4385,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4024,9 +4399,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>104</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4056,7 +4456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:11:42</t>
+          <t>Última actualización: 10:43:56</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4847,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4461,7 +4861,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4263
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E144"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:56</t>
+          <t>Última actualización: 10:59:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 139</t>
+          <t>Total filas: 150</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11:03</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,12 +3298,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11:12</t>
+          <t>11:06</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>102</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3578,16 +3578,16 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>118</v>
+        <v>21</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:21</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,23 +3923,298 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>69</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>75</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
           <t>10:43:56</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>92</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>84</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>85</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>104</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>89</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>113</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>99</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>100</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
         <is>
           <t>12:42</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C154" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D144" t="n">
-        <v>119</v>
-      </c>
-      <c r="E144" t="inlineStr">
+      <c r="D154" t="n">
+        <v>103</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>117</v>
+      </c>
+      <c r="E155" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3956,7 +4231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3969,14 +4244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:56</t>
+          <t>Última actualización: 10:59:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4385,21 +4660,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4410,23 +4685,73 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>39</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>10:43:56</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>12:27</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D23" t="n">
         <v>104</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4443,7 +4768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4456,14 +4781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:56</t>
+          <t>Última actualización: 10:59:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -4864,6 +5189,56 @@
         <v>44</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>29</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>119</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4264
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:20</t>
+          <t>Última actualización: 11:20:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 150</t>
+          <t>Total filas: 158</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:21</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>118</v>
+        <v>44</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:29</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4128,16 +4128,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,23 +4198,223 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>73</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>10:43:56</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>113</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>78</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
           <t>10:59:20</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>100</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>80</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>82</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
         <is>
           <t>12:56</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D155" t="n">
-        <v>117</v>
-      </c>
-      <c r="E155" t="inlineStr">
+      <c r="D161" t="n">
+        <v>96</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>102</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>114</v>
+      </c>
+      <c r="E163" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4244,7 +4444,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:20</t>
+          <t>Última actualización: 11:20:26</t>
         </is>
       </c>
     </row>
@@ -4660,7 +4860,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4674,7 +4874,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4685,7 +4885,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4699,7 +4899,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4735,7 +4935,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4749,7 +4949,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4781,7 +4981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:20</t>
+          <t>Última actualización: 11:20:26</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5397,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5211,7 +5411,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -5222,7 +5422,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5236,7 +5436,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4265
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E163"/>
+  <dimension ref="A1:E176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:26</t>
+          <t>Última actualización: 11:43:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 158</t>
+          <t>Total filas: 171</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,12 +3923,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>73</v>
+        <v>39</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4328,16 +4328,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,23 +4398,348 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>55</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>10:59:20</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>100</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
           <t>11:20:26</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>80</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>59</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>73</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>74</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>102</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>90</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>90</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
         <is>
           <t>13:14</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C172" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D163" t="n">
+      <c r="D172" t="n">
         <v>114</v>
       </c>
-      <c r="E163" t="inlineStr">
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>98</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>101</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>109</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>117</v>
+      </c>
+      <c r="E176" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4431,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4444,14 +4769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:26</t>
+          <t>Última actualización: 11:43:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4910,7 +5235,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4924,7 +5249,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>104</v>
+        <v>44</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4952,6 +5277,56 @@
         <v>68</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>74</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>101</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4968,7 +5343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4981,14 +5356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:20:26</t>
+          <t>Última actualización: 11:43:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -5422,25 +5797,75 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>74</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>11:20:26</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>12:58</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D23" t="n">
         <v>98</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>105</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4266
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:54</t>
+          <t>Última actualización: 11:59:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 171</t>
+          <t>Total filas: 185</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:59</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4078,16 +4078,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>92</v>
+        <v>11</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,12 +4148,12 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>38</v>
+        <v>92</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,16 +4678,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,23 +4723,373 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>58</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>59</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>11:20:26</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>102</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
           <t>11:43:54</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>90</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>74</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>75</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>98</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>101</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>86</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>89</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>11:43:54</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>109</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>94</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
         <is>
           <t>13:40</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
+      <c r="C188" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D176" t="n">
-        <v>117</v>
-      </c>
-      <c r="E176" t="inlineStr">
+      <c r="D188" t="n">
+        <v>101</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>108</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>111</v>
+      </c>
+      <c r="E190" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4756,7 +5106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4769,14 +5119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:54</t>
+          <t>Última actualización: 11:59:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5610,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5274,7 +5624,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5310,23 +5660,73 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>59</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>11:43:54</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>101</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>86</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5343,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5356,14 +5756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:54</t>
+          <t>Última actualización: 11:59:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -5822,7 +6222,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5836,7 +6236,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5866,6 +6266,56 @@
       <c r="E24" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>90</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>114</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4267
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:59:04</t>
+          <t>Última actualización: 12:17:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 185</t>
+          <t>Total filas: 192</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,12 +4548,12 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,12 +4573,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,12 +4598,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>101</v>
+        <v>56</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,16 +4928,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>108</v>
+        <v>75</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,23 +5073,198 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>76</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
           <t>11:59:04</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>94</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>83</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>90</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>92</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>11:59:04</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C195" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D190" t="n">
+      <c r="D195" t="n">
         <v>111</v>
       </c>
-      <c r="E190" t="inlineStr">
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>110</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>119</v>
+      </c>
+      <c r="E197" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5119,7 +5294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:59:04</t>
+          <t>Última actualización: 12:17:52</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5760,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5599,7 +5774,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5635,7 +5810,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5649,7 +5824,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5685,7 +5860,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5699,7 +5874,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5743,7 +5918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5756,14 +5931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:59:04</t>
+          <t>Última actualización: 12:17:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6372,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6211,7 +6386,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -6247,7 +6422,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6261,7 +6436,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6297,23 +6472,48 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>95</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>11:59:04</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>13:53</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>114</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4268
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:52</t>
+          <t>Última actualización: 12:37:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 192</t>
+          <t>Total filas: 200</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>56</v>
+        <v>102</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,12 +4923,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>11:43:54</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,12 +5098,12 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:34</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5253,18 +5253,218 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>92</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>73</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>78</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>12:17:52</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>110</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>91</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>91</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
           <t>14:16</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C203" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D197" t="n">
-        <v>119</v>
-      </c>
-      <c r="E197" t="inlineStr">
+      <c r="D203" t="n">
+        <v>99</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>109</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>111</v>
+      </c>
+      <c r="E205" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5281,7 +5481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5294,14 +5494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:52</t>
+          <t>Última actualización: 12:37:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5835,7 +6035,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5849,7 +6049,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5860,7 +6060,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5874,7 +6074,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5902,6 +6102,31 @@
         <v>86</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:37:34</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>111</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5931,7 +6156,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:52</t>
+          <t>Última actualización: 12:37:34</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6597,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6386,7 +6611,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -6447,7 +6672,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6461,7 +6686,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6472,7 +6697,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6486,7 +6711,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4269
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:34</t>
+          <t>Última actualización: 12:52:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 200</t>
+          <t>Total filas: 205</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,12 +4848,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>56</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>11:43:54</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>98</v>
+        <v>22</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,12 +5173,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13:34</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5203,16 +5203,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5228,16 +5228,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:34</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5328,16 +5328,16 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,23 +5448,148 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>76</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>84</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>94</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C208" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D205" t="n">
-        <v>111</v>
-      </c>
-      <c r="E205" t="inlineStr">
+      <c r="D208" t="n">
+        <v>96</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>109</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>116</v>
+      </c>
+      <c r="E210" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5481,7 +5606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5494,14 +5619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:34</t>
+          <t>Última actualización: 12:52:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -6035,7 +6160,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6049,7 +6174,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -6060,7 +6185,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -6074,7 +6199,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -6110,7 +6235,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6124,9 +6249,34 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>116</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6156,7 +6306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:37:34</t>
+          <t>Última actualización: 12:52:27</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6772,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6636,7 +6786,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -6672,7 +6822,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6686,7 +6836,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6722,7 +6872,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -6736,7 +6886,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>114</v>
+        <v>61</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4270
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E210"/>
+  <dimension ref="A1:E219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:27</t>
+          <t>Última actualización: 13:10:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 205</t>
+          <t>Total filas: 214</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5078,16 +5078,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,16 +5178,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5228,16 +5228,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>13:34</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,12 +5248,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:34</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:36</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>110</v>
+        <v>37</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,18 +5578,243 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>84</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>67</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>75</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>12:52:27</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>94</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>77</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>78</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>91</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
           <t>14:48</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C217" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D210" t="n">
-        <v>116</v>
-      </c>
-      <c r="E210" t="inlineStr">
+      <c r="D217" t="n">
+        <v>98</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>107</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>117</v>
+      </c>
+      <c r="E219" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5606,7 +5831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5619,14 +5844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:27</t>
+          <t>Última actualización: 13:10:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6435,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6224,7 +6449,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>86</v>
+        <v>15</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6235,7 +6460,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6249,7 +6474,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6260,7 +6485,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6274,9 +6499,34 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>107</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:52:27</t>
+          <t>Última actualización: 13:10:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -6822,7 +7072,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6836,7 +7086,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -6889,6 +7139,56 @@
         <v>61</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>45</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:10:04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>78</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4271
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:04</t>
+          <t>Última actualización: 13:37:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 214</t>
+          <t>Total filas: 221</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>58</v>
+        <v>110</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,12 +5598,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,12 +5673,12 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,23 +5798,198 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>79</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
           <t>13:10:04</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>107</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>88</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
         <is>
           <t>15:07</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr">
+      <c r="C222" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D219" t="n">
-        <v>117</v>
-      </c>
-      <c r="E219" t="inlineStr">
+      <c r="D222" t="n">
+        <v>90</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>93</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>94</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>109</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>111</v>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5831,7 +6006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5844,14 +6019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:04</t>
+          <t>Última actualización: 13:37:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6635,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6474,7 +6649,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6485,7 +6660,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6499,7 +6674,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6510,23 +6685,73 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>79</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>13:10:04</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>14:57</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>107</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>111</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6543,7 +6768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,14 +6781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:10:04</t>
+          <t>Última actualización: 13:37:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -7172,25 +7397,75 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>21</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>78</v>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D30" t="n">
+        <v>51</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:37:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>96</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4272
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:37:24</t>
+          <t>Última actualización: 13:55:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 221</t>
+          <t>Total filas: 228</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>40</v>
+        <v>84</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>109</v>
+        <v>72</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5978,18 +5978,193 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>93</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>76</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>78</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>89</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>91</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
+      <c r="C231" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D226" t="n">
+      <c r="D231" t="n">
+        <v>93</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
         <v>111</v>
       </c>
-      <c r="E226" t="inlineStr">
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>113</v>
+      </c>
+      <c r="E233" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6019,7 +6194,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:37:24</t>
+          <t>Última actualización: 13:55:18</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6810,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6649,7 +6824,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6660,7 +6835,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6674,7 +6849,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6710,7 +6885,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6724,7 +6899,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>107</v>
+        <v>62</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6735,7 +6910,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6749,7 +6924,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6768,7 +6943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6781,14 +6956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:37:24</t>
+          <t>Última actualización: 13:55:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -7397,12 +7572,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13:58</t>
+          <t>13:57</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -7411,7 +7586,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -7427,7 +7602,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -7436,7 +7611,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -7452,18 +7627,68 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:29</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>34</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>15:13</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>96</v>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="D33" t="n">
+        <v>78</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4273
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:55:18</t>
+          <t>Última actualización: 14:10:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 228</t>
+          <t>Total filas: 237</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>12:52:27</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>12:52:27</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5978,16 +5978,16 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6153,18 +6153,243 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>89</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>91</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>77</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>78</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>91</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>13:55:18</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>111</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
           <t>15:48</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr">
+      <c r="C239" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D233" t="n">
-        <v>113</v>
-      </c>
-      <c r="E233" t="inlineStr">
+      <c r="D239" t="n">
+        <v>98</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>107</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>107</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>117</v>
+      </c>
+      <c r="E242" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6194,7 +6419,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:55:18</t>
+          <t>Última actualización: 14:10:16</t>
         </is>
       </c>
     </row>
@@ -6810,7 +7035,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6824,7 +7049,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6835,7 +7060,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6849,7 +7074,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6885,7 +7110,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6899,7 +7124,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6910,7 +7135,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6924,7 +7149,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6943,7 +7168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,14 +7181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:55:18</t>
+          <t>Última actualización: 14:10:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -7622,7 +7847,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7636,7 +7861,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7672,7 +7897,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7686,11 +7911,36 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>103</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4274
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E242"/>
+  <dimension ref="A1:E250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:10:16</t>
+          <t>Última actualización: 14:32:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 237</t>
+          <t>Total filas: 245</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,12 +6123,12 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6253,16 +6253,16 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>107</v>
+        <v>76</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,23 +6373,223 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>84</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>84</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
           <t>14:10:16</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>107</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>107</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>88</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
         <is>
           <t>16:07</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr">
+      <c r="C247" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D242" t="n">
-        <v>117</v>
-      </c>
-      <c r="E242" t="inlineStr">
+      <c r="D247" t="n">
+        <v>95</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>105</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>111</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>114</v>
+      </c>
+      <c r="E250" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6419,7 +6619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:10:16</t>
+          <t>Última actualización: 14:32:21</t>
         </is>
       </c>
     </row>
@@ -7060,7 +7260,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7074,7 +7274,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -7085,7 +7285,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7099,7 +7299,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>79</v>
+        <v>24</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7135,7 +7335,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7149,7 +7349,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7181,7 +7381,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:10:16</t>
+          <t>Última actualización: 14:32:21</t>
         </is>
       </c>
     </row>
@@ -7897,7 +8097,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7911,7 +8111,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7922,7 +8122,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7936,7 +8136,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4275
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E250"/>
+  <dimension ref="A1:E256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:32:21</t>
+          <t>Última actualización: 14:51:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 245</t>
+          <t>Total filas: 251</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>13:37:24</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>13:37:24</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6173,12 +6173,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6228,16 +6228,16 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,12 +6423,12 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,12 +6473,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>105</v>
+        <v>68</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,23 +6573,173 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>76</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>86</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>92</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
           <t>16:26</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
+      <c r="C253" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D250" t="n">
-        <v>114</v>
-      </c>
-      <c r="E250" t="inlineStr">
+      <c r="D253" t="n">
+        <v>95</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>107</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>110</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>118</v>
+      </c>
+      <c r="E256" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6619,7 +6769,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:32:21</t>
+          <t>Última actualización: 14:51:27</t>
         </is>
       </c>
     </row>
@@ -7285,7 +7435,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7299,7 +7449,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7335,7 +7485,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7349,7 +7499,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7368,7 +7518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7381,14 +7531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:32:21</t>
+          <t>Última actualización: 14:51:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8247,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8111,7 +8261,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -8122,7 +8272,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8136,11 +8286,36 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>107</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4276
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E256"/>
+  <dimension ref="A1:E274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:27</t>
+          <t>Última actualización: 15:10:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 251</t>
+          <t>Total filas: 269</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,12 +6173,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,12 +6198,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>111</v>
+        <v>77</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6403,16 +6403,16 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6453,16 +6453,16 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>107</v>
+        <v>37</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,16 +6603,16 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>95</v>
+        <v>46</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,17 +6673,17 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6728,18 +6728,468 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>68</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>14:32:21</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>88</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>56</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>76</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>60</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>16:17</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>86</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>72</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>92</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>76</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>87</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>107</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>16:39</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>89</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>90</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>110</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>91</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
           <t>16:49</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr">
+      <c r="C271" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D256" t="n">
+      <c r="D271" t="n">
         <v>118</v>
       </c>
-      <c r="E256" t="inlineStr">
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>102</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>106</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>117</v>
+      </c>
+      <c r="E274" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6756,7 +7206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6769,14 +7219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:27</t>
+          <t>Última actualización: 15:10:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -7485,23 +7935,73 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>17</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>14:51:27</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>37</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>117</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7518,7 +8018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7531,14 +8031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:27</t>
+          <t>Última actualización: 15:10:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -8247,12 +8747,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -8261,7 +8761,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -8277,45 +8777,145 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>42</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>14:51:27</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>62</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>87</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>16:38</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D38" t="n">
         <v>107</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>112</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4277
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E274"/>
+  <dimension ref="A1:E286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:10:58</t>
+          <t>Última actualización: 15:47:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 269</t>
+          <t>Total filas: 281</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6523,7 +6523,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6723,12 +6723,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>68</v>
+        <v>107</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,12 +6748,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6762,7 +6762,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,12 +6848,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>16:22</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6903,16 +6903,16 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6928,16 +6928,16 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:22</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>107</v>
+        <v>38</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>16:39</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7028,16 +7028,16 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>110</v>
+        <v>51</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7078,16 +7078,16 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:39</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7128,16 +7128,16 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7178,18 +7178,318 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>91</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>14:51:27</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>118</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>102</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>66</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>69</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>15:10:58</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
           <t>17:07</t>
         </is>
       </c>
-      <c r="C274" t="inlineStr">
+      <c r="C279" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D274" t="n">
+      <c r="D279" t="n">
         <v>117</v>
       </c>
-      <c r="E274" t="inlineStr">
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>81</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>89</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>95</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>105</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>106</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>109</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>111</v>
+      </c>
+      <c r="E286" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7206,7 +7506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7219,14 +7519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:10:58</t>
+          <t>Última actualización: 15:47:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -8002,6 +8302,56 @@
         <v>117</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>81</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>105</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8018,7 +8368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8031,14 +8381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:10:58</t>
+          <t>Última actualización: 15:47:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8822,7 +9172,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8836,7 +9186,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -8872,7 +9222,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8886,7 +9236,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>107</v>
+        <v>51</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -8914,6 +9264,31 @@
         <v>112</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>15:47:31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>76</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4278
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E286"/>
+  <dimension ref="A1:E291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:31</t>
+          <t>Última actualización: 16:04:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 281</t>
+          <t>Total filas: 286</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7037,7 +7037,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>102</v>
+        <v>48</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7353,16 +7353,16 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7378,16 +7378,16 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7453,16 +7453,16 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,23 +7473,148 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>92</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>93</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>94</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
           <t>15:47:31</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B289" t="inlineStr">
         <is>
           <t>17:38</t>
         </is>
       </c>
-      <c r="C286" t="inlineStr">
+      <c r="C289" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D286" t="n">
+      <c r="D289" t="n">
         <v>111</v>
       </c>
-      <c r="E286" t="inlineStr">
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>17:49</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>105</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>115</v>
+      </c>
+      <c r="E291" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7506,7 +7631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7519,14 +7644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:31</t>
+          <t>Última actualización: 16:04:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8410,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8299,7 +8424,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -8335,7 +8460,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8349,9 +8474,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>115</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8381,7 +8531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:47:31</t>
+          <t>Última actualización: 16:04:56</t>
         </is>
       </c>
     </row>
@@ -9197,7 +9347,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -9211,7 +9361,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -9247,7 +9397,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9261,7 +9411,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>112</v>
+        <v>58</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4279
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E291"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:56</t>
+          <t>Última actualización: 16:28:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 286</t>
+          <t>Total filas: 295</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7412,7 +7412,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7528,16 +7528,16 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7578,16 +7578,16 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,23 +7598,248 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>75</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
           <t>16:04:56</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr">
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>17:49</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>105</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>82</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>85</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>16:04:56</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
         <is>
           <t>17:59</t>
         </is>
       </c>
-      <c r="C291" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D291" t="n">
+      <c r="D295" t="n">
         <v>115</v>
       </c>
-      <c r="E291" t="inlineStr">
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>97</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>100</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>102</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>112</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>115</v>
+      </c>
+      <c r="E300" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7631,7 +7856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7644,14 +7869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:56</t>
+          <t>Última actualización: 16:28:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8435,7 +8660,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8449,7 +8674,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -8460,7 +8685,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8474,7 +8699,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8485,23 +8710,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>85</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>16:04:56</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>17:59</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>115</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>115</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8518,7 +8793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8531,14 +8806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:04:56</t>
+          <t>Última actualización: 16:28:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -9347,12 +9622,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:29</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -9361,7 +9636,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -9372,12 +9647,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -9386,7 +9661,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -9397,48 +9672,73 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>58</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>17:03</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>76</v>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D41" t="n">
+        <v>35</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4280
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:24</t>
+          <t>Última actualización: 16:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 295</t>
+          <t>Total filas: 301</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>48</v>
+        <v>118</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,12 +7248,12 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,12 +7348,12 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>106</v>
+        <v>49</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,12 +7548,12 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,12 +7598,12 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -7612,7 +7612,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7753,16 +7753,16 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,23 +7823,173 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>85</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>87</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>97</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>99</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
           <t>16:28:24</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
+      <c r="B304" t="inlineStr">
         <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr">
+      <c r="C304" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D300" t="n">
+      <c r="D304" t="n">
         <v>115</v>
       </c>
-      <c r="E300" t="inlineStr">
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>112</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>114</v>
+      </c>
+      <c r="E306" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7856,7 +8006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7869,14 +8019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:24</t>
+          <t>Última actualización: 16:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -8635,7 +8785,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8649,7 +8799,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -8685,7 +8835,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8699,7 +8849,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8710,12 +8860,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -8724,7 +8874,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -8735,12 +8885,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -8749,7 +8899,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8760,23 +8910,73 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D40" t="n">
         <v>115</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:28:24</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>115</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8793,7 +8993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8806,14 +9006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:28:24</t>
+          <t>Última actualización: 16:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -9697,7 +9897,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -9711,7 +9911,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -9739,6 +9939,31 @@
         <v>35</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:43:37</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>106</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4281
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E306"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:37</t>
+          <t>Última actualización: 16:56:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 301</t>
+          <t>Total filas: 306</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,12 +7373,12 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7478,16 +7478,16 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,12 +7498,12 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>106</v>
+        <v>35</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7603,16 +7603,16 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,12 +7623,12 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,16 +7703,16 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,12 +7773,12 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7787,7 +7787,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>115</v>
+        <v>84</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7953,16 +7953,16 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,23 +7973,148 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>87</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>88</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>89</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>99</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C306" t="inlineStr">
+      <c r="C310" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D306" t="n">
-        <v>114</v>
-      </c>
-      <c r="E306" t="inlineStr">
+      <c r="D310" t="n">
+        <v>101</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>117</v>
+      </c>
+      <c r="E311" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8019,7 +8144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:37</t>
+          <t>Última actualización: 16:56:33</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8935,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8824,7 +8949,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -8835,7 +8960,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8849,7 +8974,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8885,7 +9010,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8899,7 +9024,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8960,7 +9085,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8974,7 +9099,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8993,7 +9118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9006,14 +9131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:43:37</t>
+          <t>Última actualización: 16:56:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9922,7 +10047,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9936,7 +10061,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9964,6 +10089,31 @@
         <v>106</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>94</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4282
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E311"/>
+  <dimension ref="A1:E321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:56:33</t>
+          <t>Última actualización: 17:12:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 306</t>
+          <t>Total filas: 316</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>106</v>
+        <v>36</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,12 +7698,12 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7778,16 +7778,16 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,17 +7848,17 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7928,16 +7928,16 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,17 +8048,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8103,18 +8103,268 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>88</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>89</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>18:27</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>75</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>78</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>16:56:33</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>99</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>84</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>85</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>98</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
           <t>18:53</t>
         </is>
       </c>
-      <c r="C311" t="inlineStr">
+      <c r="C319" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D311" t="n">
-        <v>117</v>
-      </c>
-      <c r="E311" t="inlineStr">
+      <c r="D319" t="n">
+        <v>101</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>113</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>116</v>
+      </c>
+      <c r="E321" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8131,7 +8381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8144,14 +8394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:56:33</t>
+          <t>Última actualización: 17:12:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -8985,21 +9235,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -9010,12 +9260,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -9024,7 +9274,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -9035,12 +9285,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -9049,7 +9299,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>41</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -9060,21 +9310,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9085,23 +9335,73 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>99</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>87</v>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D43" t="n">
+        <v>71</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>116</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9118,7 +9418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9131,14 +9431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:56:33</t>
+          <t>Última actualización: 17:12:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -10097,7 +10397,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10111,11 +10411,36 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>110</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4283
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:08</t>
+          <t>Última actualización: 17:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 316</t>
+          <t>Total filas: 326</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,12 +7773,12 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7787,7 +7787,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:43:37</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>17:49</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,12 +7823,12 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:49</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,12 +7873,12 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7887,7 +7887,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,12 +7898,12 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7912,7 +7912,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>115</v>
+        <v>41</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8003,16 +8003,16 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8178,16 +8178,16 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8203,16 +8203,16 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8253,16 +8253,16 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8278,16 +8278,16 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8328,16 +8328,16 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,23 +8348,273 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>59</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
           <t>17:12:08</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>98</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>75</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>86</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>113</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>89</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>17:12:08</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
         <is>
           <t>19:08</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr">
+      <c r="C327" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D321" t="n">
+      <c r="D327" t="n">
         <v>116</v>
       </c>
-      <c r="E321" t="inlineStr">
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>96</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>98</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>103</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>104</v>
+      </c>
+      <c r="E331" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8381,7 +8631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8394,14 +8644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:08</t>
+          <t>Última actualización: 17:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -9260,7 +9510,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9274,7 +9524,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -9335,7 +9585,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:43:37</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9349,7 +9599,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>99</v>
+        <v>44</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -9385,23 +9635,73 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>89</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>17:12:08</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>19:08</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>116</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>104</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9418,7 +9718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9431,14 +9731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:12:08</t>
+          <t>Última actualización: 17:38:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -10422,23 +10722,73 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>54</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>83</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>17:12:08</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D46" t="n">
         <v>110</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4284
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E331"/>
+  <dimension ref="A1:E338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:53</t>
+          <t>Última actualización: 17:54:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 326</t>
+          <t>Total filas: 333</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>115</v>
+        <v>17</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>27</v>
+        <v>115</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,12 +7998,12 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>18:19</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,12 +8098,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -8112,7 +8112,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,12 +8173,12 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -8187,7 +8187,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>47</v>
+        <v>88</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,12 +8248,12 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8278,16 +8278,16 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,12 +8323,12 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>113</v>
+        <v>61</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8478,16 +8478,16 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>116</v>
+        <v>71</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8578,16 +8578,16 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8603,18 +8603,193 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>98</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>83</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>84</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>87</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
           <t>19:22</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr">
+      <c r="C335" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D331" t="n">
-        <v>104</v>
-      </c>
-      <c r="E331" t="inlineStr">
+      <c r="D335" t="n">
+        <v>88</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>106</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>107</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>109</v>
+      </c>
+      <c r="E338" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8631,7 +8806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8644,14 +8819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:53</t>
+          <t>Última actualización: 17:54:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -9560,12 +9735,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -9574,7 +9749,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9585,21 +9760,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -9610,12 +9785,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -9624,7 +9799,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9635,21 +9810,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9660,12 +9835,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -9674,7 +9849,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>116</v>
+        <v>73</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9685,23 +9860,48 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>116</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>19:22</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>104</v>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D47" t="n">
+        <v>88</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9718,7 +9918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9731,14 +9931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:53</t>
+          <t>Última actualización: 17:54:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -10747,48 +10947,98 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>17:38:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>83</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>17:12:08</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D47" t="n">
         <v>110</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17:54:37</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>71</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4285
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E338"/>
+  <dimension ref="A1:E342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:37</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 333</t>
+          <t>Total filas: 337</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8073,7 +8073,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -8087,7 +8087,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -8162,7 +8162,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8198,7 +8198,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -8212,7 +8212,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8248,7 +8248,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8373,7 +8373,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -8387,7 +8387,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,7 +8398,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,7 +8448,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -8462,7 +8462,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8512,7 +8512,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8728,16 +8728,16 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,23 +8773,123 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>90</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>91</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
           <t>17:54:37</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
+      <c r="B340" t="inlineStr">
         <is>
           <t>19:43</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
+      <c r="C340" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D338" t="n">
+      <c r="D340" t="n">
         <v>109</v>
       </c>
-      <c r="E338" t="inlineStr">
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>19:57</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>107</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>112</v>
+      </c>
+      <c r="E342" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8806,7 +8906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8819,14 +8919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:37</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9910,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -9824,7 +9924,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9860,7 +9960,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9874,7 +9974,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9902,6 +10002,31 @@
         <v>88</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>73</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9918,7 +10043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9931,14 +10056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:37</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -10972,37 +11097,37 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>19:02</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -11011,7 +11136,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -11022,25 +11147,75 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>52</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>17:54:37</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>19:05</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
         <v>71</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>112</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4286
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E342"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 337</t>
+          <t>Total filas: 344</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8373,7 +8373,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -8387,7 +8387,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,7 +8398,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8512,7 +8512,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8537,7 +8537,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8573,12 +8573,12 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>17:38:53</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,12 +8623,12 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8653,16 +8653,16 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,12 +8673,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>17:54:37</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8687,7 +8687,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,12 +8748,12 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -8762,7 +8762,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8778,16 +8778,16 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:32</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>107</v>
+        <v>69</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,23 +8873,198 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>71</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>84</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
           <t>18:10:26</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>19:57</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>107</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>89</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
         <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C346" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D342" t="n">
-        <v>112</v>
-      </c>
-      <c r="E342" t="inlineStr">
+      <c r="D346" t="n">
+        <v>90</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>90</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>110</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>113</v>
+      </c>
+      <c r="E349" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8906,7 +9081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8919,14 +9094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -9935,7 +10110,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9949,7 +10124,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9985,7 +10160,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:54:37</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9999,7 +10174,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -10027,6 +10202,31 @@
         <v>73</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10043,7 +10243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10056,14 +10256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -11097,7 +11297,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -11111,7 +11311,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -11122,7 +11322,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:38:53</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11136,7 +11336,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -11197,23 +11397,48 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>18:32:38</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>89</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>18:10:26</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
         <v>112</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4287
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:32:38</t>
+          <t>Última actualización: 18:50:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 344</t>
+          <t>Total filas: 349</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -8398,7 +8398,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8512,7 +8512,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,7 +8573,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,12 +8798,12 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>19:32</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -8812,7 +8812,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8828,16 +8828,16 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:32</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>84</v>
+        <v>53</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9053,18 +9053,143 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>90</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>73</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>92</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
           <t>20:25</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C352" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D349" t="n">
-        <v>113</v>
-      </c>
-      <c r="E349" t="inlineStr">
+      <c r="D352" t="n">
+        <v>95</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>111</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>115</v>
+      </c>
+      <c r="E354" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9081,7 +9206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9094,14 +9219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:32:38</t>
+          <t>Última actualización: 18:50:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -10135,7 +10260,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10149,7 +10274,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -10185,7 +10310,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10199,7 +10324,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -10227,6 +10352,56 @@
         <v>90</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>73</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>111</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10243,7 +10418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10256,14 +10431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:32:38</t>
+          <t>Última actualización: 18:50:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -11397,48 +11572,98 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>89</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D52" t="n">
+        <v>72</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>18:50:27</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
         <v>112</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4288
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E354"/>
+  <dimension ref="A1:E359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:50:27</t>
+          <t>Última actualización: 19:08:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 349</t>
+          <t>Total filas: 354</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,7 +8573,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8773,7 +8773,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,12 +8973,12 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -8987,7 +8987,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9028,16 +9028,16 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9153,16 +9153,16 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,23 +9173,148 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>75</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>77</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>93</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
+      <c r="C357" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D354" t="n">
+      <c r="D357" t="n">
+        <v>97</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>108</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
         <v>115</v>
       </c>
-      <c r="E354" t="inlineStr">
+      <c r="E359" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9219,7 +9344,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:50:27</t>
+          <t>Última actualización: 19:08:25</t>
         </is>
       </c>
     </row>
@@ -10260,7 +10385,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10274,7 +10399,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -10310,7 +10435,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10324,7 +10449,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -10360,7 +10485,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10374,7 +10499,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -10385,7 +10510,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10399,7 +10524,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -10431,7 +10556,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:50:27</t>
+          <t>Última actualización: 19:08:25</t>
         </is>
       </c>
     </row>
@@ -11572,7 +11697,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -11586,7 +11711,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -11622,7 +11747,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -11636,7 +11761,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -11647,7 +11772,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -11661,7 +11786,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4289
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E359"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:08:25</t>
+          <t>Última actualización: 19:33:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 354</t>
+          <t>Total filas: 363</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8858,11 +8858,11 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8878,16 +8878,16 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,12 +8973,12 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -8987,7 +8987,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:32:38</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>68</v>
+        <v>107</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>18:50:27</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9112,7 +9112,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>90</v>
+        <v>29</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,21 +9148,21 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>18:50:27</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,12 +9173,12 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9203,16 +9203,16 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,21 +9223,21 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9253,16 +9253,16 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,21 +9273,21 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>108</v>
+        <v>63</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,23 +9298,248 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>68</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>71</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
           <t>19:08:25</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>97</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>78</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>108</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>88</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>89</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>19:08:25</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
         <is>
           <t>21:03</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C366" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D359" t="n">
+      <c r="D366" t="n">
         <v>115</v>
       </c>
-      <c r="E359" t="inlineStr">
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>96</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>113</v>
+      </c>
+      <c r="E368" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9344,7 +9569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:08:25</t>
+          <t>Última actualización: 19:33:46</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10685,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10474,7 +10699,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>90</v>
+        <v>29</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -10510,7 +10735,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10524,7 +10749,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -10556,7 +10781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:08:25</t>
+          <t>Última actualización: 19:33:46</t>
         </is>
       </c>
     </row>
@@ -11722,7 +11947,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -11736,7 +11961,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -11772,7 +11997,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -11786,7 +12011,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4290
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:46</t>
+          <t>Última actualización: 19:52:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 363</t>
+          <t>Total filas: 371</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:32:38</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9012,7 +9012,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -9123,7 +9123,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -9133,11 +9133,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,12 +9148,12 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -9162,7 +9162,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9228,16 +9228,16 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,21 +9248,21 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>77</v>
+        <v>31</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9278,16 +9278,16 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,21 +9298,21 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,21 +9348,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,21 +9373,21 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9398,21 +9398,21 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9453,16 +9453,16 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,18 +9528,218 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>88</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>70</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>89</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>71</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>19:33:46</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>96</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>78</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C374" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D368" t="n">
-        <v>113</v>
-      </c>
-      <c r="E368" t="inlineStr">
+      <c r="D374" t="n">
+        <v>94</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>102</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>114</v>
+      </c>
+      <c r="E376" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9556,7 +9756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9569,14 +9769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:46</t>
+          <t>Última actualización: 19:52:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -10710,7 +10910,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10724,7 +10924,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -10752,6 +10952,31 @@
         <v>68</v>
       </c>
       <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>50</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10768,7 +10993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10781,14 +11006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:33:46</t>
+          <t>Última actualización: 19:52:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -11972,7 +12197,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -11986,7 +12211,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -12014,6 +12239,31 @@
         <v>69</v>
       </c>
       <c r="E53" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>19:52:02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>52</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4291
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E376"/>
+  <dimension ref="A1:E379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:03</t>
+          <t>Última actualización: 20:09:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 371</t>
+          <t>Total filas: 374</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8858,11 +8858,11 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,7 +8873,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -8883,11 +8883,11 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -9133,11 +9133,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9248,7 +9248,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -9262,7 +9262,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -9312,7 +9312,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9337,7 +9337,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9387,7 +9387,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -9437,7 +9437,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -9462,7 +9462,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9523,12 +9523,12 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -9537,7 +9537,7 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,12 +9548,12 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -9562,7 +9562,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,7 +9573,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -9583,11 +9583,11 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,12 +9598,12 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -9612,7 +9612,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9623,21 +9623,21 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9648,12 +9648,12 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -9662,7 +9662,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,21 +9673,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,23 +9723,98 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>85</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>20:09:11</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>21:38</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>89</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>20:09:11</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>91</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>20:09:11</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C376" t="inlineStr">
+      <c r="C379" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D376" t="n">
-        <v>114</v>
-      </c>
-      <c r="E376" t="inlineStr">
+      <c r="D379" t="n">
+        <v>97</v>
+      </c>
+      <c r="E379" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9769,7 +9844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:03</t>
+          <t>Última actualización: 20:09:11</t>
         </is>
       </c>
     </row>
@@ -10960,7 +11035,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10974,7 +11049,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -10993,7 +11068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11006,14 +11081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:03</t>
+          <t>Última actualización: 20:09:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -12264,6 +12339,56 @@
         <v>52</v>
       </c>
       <c r="E54" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20:09:11</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:47</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>38</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20:09:11</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>77</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4292
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E379"/>
+  <dimension ref="A1:E382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:11</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 374</t>
+          <t>Total filas: 377</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:08:42</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:08:42</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8858,11 +8858,11 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,7 +8873,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -8883,11 +8883,11 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -9158,11 +9158,11 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9337,7 +9337,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,7 +9348,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -9437,7 +9437,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -9462,7 +9462,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9523,7 +9523,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -9537,7 +9537,7 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -9637,7 +9637,7 @@
         </is>
       </c>
       <c r="D372" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -9687,7 +9687,7 @@
         </is>
       </c>
       <c r="D374" t="n">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,7 +9698,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,7 +9723,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -9737,7 +9737,7 @@
         </is>
       </c>
       <c r="D376" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,12 +9748,12 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -9762,7 +9762,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9778,16 +9778,16 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9798,23 +9798,98 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>69</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr">
+      <c r="C380" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D379" t="n">
-        <v>97</v>
-      </c>
-      <c r="E379" t="inlineStr">
+      <c r="D380" t="n">
+        <v>75</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>93</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>100</v>
+      </c>
+      <c r="E382" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9844,7 +9919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:11</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
@@ -11010,7 +11085,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -11024,7 +11099,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -11068,7 +11143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11081,14 +11156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:11</t>
+          <t>Última actualización: 20:31:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -12372,25 +12447,75 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>17</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>77</v>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D57" t="n">
+        <v>55</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>105</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4293
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E382"/>
+  <dimension ref="A1:E393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:49:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 377</t>
+          <t>Total filas: 388</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8858,11 +8858,11 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,7 +8873,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -8883,11 +8883,11 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -9123,7 +9123,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -9133,11 +9133,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -9158,11 +9158,11 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9473,7 +9473,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -9487,7 +9487,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,7 +9498,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -9512,7 +9512,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>108</v>
+        <v>7</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9598,7 +9598,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -9612,7 +9612,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9648,7 +9648,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -9662,7 +9662,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:17</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9753,16 +9753,16 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9773,12 +9773,12 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -9787,7 +9787,7 @@
         </is>
       </c>
       <c r="D378" t="n">
-        <v>89</v>
+        <v>46</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9803,16 +9803,16 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,21 +9823,21 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9848,21 +9848,21 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9878,18 +9878,293 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>69</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>54</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>56</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>75</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>22:03</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>74</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>93</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>22:06</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>77</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>81</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>20:31:19</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
           <t>22:11</t>
         </is>
       </c>
-      <c r="C382" t="inlineStr">
+      <c r="C390" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D382" t="n">
+      <c r="D390" t="n">
         <v>100</v>
       </c>
-      <c r="E382" t="inlineStr">
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>104</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>114</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>22:47</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>118</v>
+      </c>
+      <c r="E393" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9906,7 +10181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9919,14 +10194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:49:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -11127,6 +11402,31 @@
         <v>33</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>104</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11143,7 +11443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11156,14 +11456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:19</t>
+          <t>Última actualización: 20:49:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -12472,12 +12772,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -12486,7 +12786,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -12497,23 +12797,73 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>37</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>86</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>20:31:19</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>22:16</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D58" t="n">
+      <c r="D60" t="n">
         <v>105</v>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4294
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E393"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:54</t>
+          <t>Última actualización: 20:59:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 388</t>
+          <t>Total filas: 393</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:08:25</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>19:08:25</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -9133,11 +9133,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -9158,11 +9158,11 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9183,7 +9183,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D355" t="n">
@@ -9648,21 +9648,21 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,12 +9673,12 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -9687,7 +9687,7 @@
         </is>
       </c>
       <c r="D374" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>21:17</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:17</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9773,21 +9773,21 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9803,16 +9803,16 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,12 +9823,12 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>20:09:11</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -9837,7 +9837,7 @@
         </is>
       </c>
       <c r="D380" t="n">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9848,21 +9848,21 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,21 +9873,21 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:09:11</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9898,21 +9898,21 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>21:43</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="E383" t="inlineStr">
         <is>
@@ -9923,21 +9923,21 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,21 +9948,21 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:43</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -9973,21 +9973,21 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>22:03</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -10003,16 +10003,16 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10023,21 +10023,21 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>22:06</t>
+          <t>22:03</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,21 +10048,21 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>22:10</t>
+          <t>22:04</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10073,21 +10073,21 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>20:31:19</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>22:11</t>
+          <t>22:06</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10098,21 +10098,21 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10123,21 +10123,21 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:31:19</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>22:43</t>
+          <t>22:11</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,23 +10148,148 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>76</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>94</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>94</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
           <t>20:49:54</t>
         </is>
       </c>
-      <c r="B393" t="inlineStr">
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>114</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>106</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>20:49:54</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
         <is>
           <t>22:47</t>
         </is>
       </c>
-      <c r="C393" t="inlineStr">
+      <c r="C398" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D393" t="n">
+      <c r="D398" t="n">
         <v>118</v>
       </c>
-      <c r="E393" t="inlineStr">
+      <c r="E398" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10194,7 +10319,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:54</t>
+          <t>Última actualización: 20:59:55</t>
         </is>
       </c>
     </row>
@@ -11410,7 +11535,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -11424,7 +11549,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -11443,7 +11568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11456,14 +11581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:54</t>
+          <t>Última actualización: 20:59:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -12797,12 +12922,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12811,7 +12936,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12827,43 +12952,68 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>22:15</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>76</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>20:31:19</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>22:16</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="D61" t="n">
         <v>105</v>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4295
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:55</t>
+          <t>Última actualización: 22:17:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 393</t>
+          <t>Total filas: 402</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>06:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:34:33</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:49:51</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:49:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>09:36:56</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:36:56</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:32:21</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>14:32:21</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>13:55:18</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>13:55:18</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6233,11 +6233,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:56:33</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:56:33</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9573,7 +9573,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>20:49:54</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -9583,11 +9583,11 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,7 +9598,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -9608,11 +9608,11 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -10173,21 +10173,21 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>20:59:55</t>
+          <t>22:17:57</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:29</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>94</v>
+        <v>12</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10198,12 +10198,12 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>20:59:55</t>
+          <t>22:17:57</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:29</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="D395" t="n">
-        <v>94</v>
+        <v>12</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -10223,21 +10223,21 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>20:49:54</t>
+          <t>20:59:55</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>22:43</t>
+          <t>22:33</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -10248,21 +10248,21 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>20:59:55</t>
+          <t>22:17:57</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>22:33</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>106</v>
+        <v>16</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -10273,23 +10273,248 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>18</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>26</v>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>20:59:55</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>106</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
           <t>20:49:54</t>
         </is>
       </c>
-      <c r="B398" t="inlineStr">
+      <c r="B401" t="inlineStr">
         <is>
           <t>22:47</t>
         </is>
       </c>
-      <c r="C398" t="inlineStr">
+      <c r="C401" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D398" t="n">
+      <c r="D401" t="n">
         <v>118</v>
       </c>
-      <c r="E398" t="inlineStr">
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>23:03</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>46</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>23:09</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>52</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>23:18</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>61</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>23:35</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>78</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>82</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>23:59</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>102</v>
+      </c>
+      <c r="E407" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10306,7 +10531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10319,14 +10544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:55</t>
+          <t>Última actualización: 22:17:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11760,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>20:59:55</t>
+          <t>22:17:57</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -11549,9 +11774,34 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>82</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11568,7 +11818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11581,14 +11831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:59:55</t>
+          <t>Última actualización: 22:17:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -13014,6 +13264,31 @@
         <v>105</v>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>22:17:57</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>22:17</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4296
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-15.xlsx
+++ b/data/horarios-141-2026-08-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:17:57</t>
+          <t>Última actualización: 23:34:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 402</t>
+          <t>Total filas: 403</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:52:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:52:27</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:02:21</t>
+          <t>07:10:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:10:54</t>
+          <t>06:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:59:52</t>
+          <t>08:30:35</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2683,11 +2683,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:30:35</t>
+          <t>08:59:52</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:11:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:11:42</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>10:43:56</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:43:56</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:20:26</t>
+          <t>10:59:20</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:20</t>
+          <t>11:20:26</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4833,11 +4833,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4858,11 +4858,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:52</t>
+          <t>13:10:04</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>13:10:04</t>
+          <t>12:17:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:37:34</t>
+          <t>11:59:04</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:59:04</t>
+          <t>12:37:34</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6348,7 +6348,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>15:10:58</t>
+          <t>14:10:16</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6358,11 +6358,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,7 +6373,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:10:16</t>
+          <t>15:10:58</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6383,11 +6383,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>14:51:27</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>14:51:27</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:04:56</t>
+          <t>16:28:24</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:28:24</t>
+          <t>16:04:56</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:12:08</t>
+          <t>15:47:31</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>15:47:31</t>
+          <t>17:12:08</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:33:46</t>
+          <t>19:52:02</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:52:02</t>
+          <t>19:33:46</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -9158,11 +9158,11 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -10183,7 +10183,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D394" t="n">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D395" t="n">
@@ -10448,7 +10448,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>22:17:57</t>
+          <t>23:34:59</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -10462,7 +10462,7 @@
         </is>
       </c>
       <c r="D405" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10473,7 +10473,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>22:17:57</t>
+          <t>23:34:59</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -10487,7 +10487,7 @@
         </is>
       </c>
       <c r="D406" t="n">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -10498,23 +10498,48 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
+          <t>23:34:59</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>23:58</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>24</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
           <t>22:17:57</t>
         </is>
       </c>
-      <c r="B407" t="inlineStr">
+      <c r="B408" t="inlineStr">
         <is>
           <t>23:59</t>
         </is>
       </c>
-      <c r="C407" t="inlineStr">
+      <c r="C408" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D407" t="n">
+      <c r="D408" t="n">
         <v>102</v>
       </c>
-      <c r="E407" t="inlineStr">
+      <c r="E408" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10544,7 +10569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:17:57</t>
+          <t>Última actualización: 23:34:59</t>
         </is>
       </c>
     </row>
@@ -11785,7 +11810,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>22:17:57</t>
+          <t>23:34:59</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -11799,7 +11824,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -11831,7 +11856,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 22:17:57</t>
+          <t>Última actualización: 23:34:59</t>
         </is>
       </c>
     </row>

</xml_diff>